<commit_message>
Templates with the new database layout
</commit_message>
<xml_diff>
--- a/inputdata/inputdata_grid.xlsx
+++ b/inputdata/inputdata_grid.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Itahisa\Desktop\pvlite\inputdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AB37533-4729-4D4B-9F3A-760A7741188A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56BD259A-3A11-4ED0-87C2-ED7691FD01DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="833" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="833" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Site" sheetId="6" r:id="rId1"/>
@@ -1179,9 +1179,6 @@
     <t>Use_Database_PV</t>
   </si>
   <si>
-    <t>N_modules</t>
-  </si>
-  <si>
     <t>Use_Database_Inv</t>
   </si>
   <si>
@@ -1216,6 +1213,9 @@
   </si>
   <si>
     <t>Set to 2 to use PVlite database (1 = Manual Mode, 2 = Use Database)</t>
+  </si>
+  <si>
+    <t>N_Modules</t>
   </si>
 </sst>
 </file>
@@ -9077,7 +9077,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="22" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C10" s="86">
         <v>25</v>
@@ -9094,7 +9094,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C11" s="20"/>
       <c r="D11" s="23" t="s">
@@ -9801,7 +9801,7 @@
       </c>
       <c r="D4" s="110"/>
       <c r="E4" s="109" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F4" s="109"/>
       <c r="G4" s="109"/>
@@ -9844,7 +9844,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="109" t="s">
-        <v>293</v>
+        <v>305</v>
       </c>
       <c r="C6" s="110">
         <v>4</v>
@@ -10203,14 +10203,14 @@
         <v>1</v>
       </c>
       <c r="B4" s="109" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C4" s="110">
         <v>1</v>
       </c>
       <c r="D4" s="110"/>
       <c r="E4" s="109" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.4">
@@ -10218,7 +10218,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="109" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C5" s="111" t="s">
         <v>260</v>
@@ -10832,14 +10832,14 @@
         <v>1</v>
       </c>
       <c r="B4" s="109" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C4" s="110">
         <v>1</v>
       </c>
       <c r="D4" s="110"/>
       <c r="E4" s="109" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.4">
@@ -10847,7 +10847,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="109" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C5" s="111" t="s">
         <v>262</v>
@@ -10862,7 +10862,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="109" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C6" s="110">
         <v>4</v>
@@ -11064,7 +11064,7 @@
         <v>15</v>
       </c>
       <c r="B18" s="105" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C18" s="108">
         <v>0</v>
@@ -11081,7 +11081,7 @@
         <v>16</v>
       </c>
       <c r="B19" s="105" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C19" s="108">
         <v>45</v>
@@ -11098,7 +11098,7 @@
         <v>17</v>
       </c>
       <c r="B20" s="105" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C20" s="108">
         <v>-20</v>
@@ -11115,7 +11115,7 @@
         <v>18</v>
       </c>
       <c r="B21" s="105" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C21" s="108">
         <v>60</v>

</xml_diff>

<commit_message>
Changing some values in templates with the new database layout
</commit_message>
<xml_diff>
--- a/inputdata/inputdata_grid.xlsx
+++ b/inputdata/inputdata_grid.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Itahisa\Desktop\pvlite\inputdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56BD259A-3A11-4ED0-87C2-ED7691FD01DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7968E01C-64E6-49C0-A713-F7B231CEE0CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="833" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9096,7 +9096,9 @@
       <c r="B11" s="22" t="s">
         <v>303</v>
       </c>
-      <c r="C11" s="20"/>
+      <c r="C11" s="20">
+        <v>0</v>
+      </c>
       <c r="D11" s="23" t="s">
         <v>7</v>
       </c>

</xml_diff>